<commit_message>
Refactor Save function to handle multiple data types and update AddAvaliador to include sigla field
</commit_message>
<xml_diff>
--- a/Execelteste/BaseAvaliador.xlsx
+++ b/Execelteste/BaseAvaliador.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1028" uniqueCount="340">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1010" uniqueCount="324">
   <si>
     <t>TimeStamp</t>
   </si>
@@ -732,250 +732,202 @@
     <t>teste107@al.insper.edu.br</t>
   </si>
   <si>
+    <t>Avaliador</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Sigla</t>
+  </si>
+  <si>
     <t>Avaliador 1</t>
   </si>
   <si>
+    <t>avaliador1@teste.com</t>
+  </si>
+  <si>
     <t>A1</t>
   </si>
   <si>
-    <t>BC</t>
-  </si>
-  <si>
-    <t>avaliador1@teste.com</t>
-  </si>
-  <si>
     <t>Avaliador 2</t>
   </si>
   <si>
+    <t>avaliador2@teste.com</t>
+  </si>
+  <si>
     <t>A2</t>
   </si>
   <si>
-    <t>BT</t>
-  </si>
-  <si>
-    <t>avaliador2@teste.com</t>
-  </si>
-  <si>
     <t>Avaliador 3</t>
   </si>
   <si>
+    <t>avaliador3@teste.com</t>
+  </si>
+  <si>
     <t>A3</t>
   </si>
   <si>
-    <t>BV</t>
-  </si>
-  <si>
-    <t>avaliador3@teste.com</t>
-  </si>
-  <si>
     <t>Avaliador 4</t>
   </si>
   <si>
+    <t>avaliador4@teste.com</t>
+  </si>
+  <si>
     <t>A4</t>
   </si>
   <si>
-    <t>CC</t>
-  </si>
-  <si>
-    <t>avaliador4@teste.com</t>
-  </si>
-  <si>
     <t>Avaliador 5</t>
   </si>
   <si>
+    <t>avaliador5@teste.com</t>
+  </si>
+  <si>
     <t>A5</t>
   </si>
   <si>
-    <t>CG</t>
-  </si>
-  <si>
-    <t>avaliador5@teste.com</t>
-  </si>
-  <si>
     <t>Avaliador 6</t>
   </si>
   <si>
+    <t>avaliador6@teste.com</t>
+  </si>
+  <si>
     <t>A6</t>
   </si>
   <si>
-    <t>FB</t>
-  </si>
-  <si>
-    <t>avaliador6@teste.com</t>
-  </si>
-  <si>
     <t>Avaliador 7</t>
   </si>
   <si>
+    <t>avaliador7@teste.com</t>
+  </si>
+  <si>
     <t>A7</t>
   </si>
   <si>
-    <t>FO</t>
-  </si>
-  <si>
-    <t>avaliador7@teste.com</t>
-  </si>
-  <si>
     <t>Avaliador 8</t>
   </si>
   <si>
+    <t>avaliador8@teste.com</t>
+  </si>
+  <si>
     <t>A8</t>
   </si>
   <si>
-    <t>GD</t>
-  </si>
-  <si>
-    <t>avaliador8@teste.com</t>
-  </si>
-  <si>
     <t>Avaliador 9</t>
   </si>
   <si>
+    <t>avaliador9@teste.com</t>
+  </si>
+  <si>
     <t>A9</t>
   </si>
   <si>
-    <t>HJ</t>
-  </si>
-  <si>
-    <t>avaliador9@teste.com</t>
-  </si>
-  <si>
     <t>Avaliador 10</t>
   </si>
   <si>
+    <t>avaliador10@teste.com</t>
+  </si>
+  <si>
     <t>A10</t>
   </si>
   <si>
-    <t>IC</t>
-  </si>
-  <si>
-    <t>avaliador10@teste.com</t>
-  </si>
-  <si>
     <t>Avaliador 11</t>
   </si>
   <si>
+    <t>avaliador11@teste.com</t>
+  </si>
+  <si>
     <t>A11</t>
   </si>
   <si>
-    <t>MC</t>
-  </si>
-  <si>
-    <t>avaliador11@teste.com</t>
-  </si>
-  <si>
     <t>Avaliador 12</t>
   </si>
   <si>
+    <t>avaliador12@teste.com</t>
+  </si>
+  <si>
     <t>A12</t>
   </si>
   <si>
-    <t>MS</t>
-  </si>
-  <si>
-    <t>avaliador12@teste.com</t>
-  </si>
-  <si>
     <t>Avaliador 13</t>
   </si>
   <si>
+    <t>avaliador13@teste.com</t>
+  </si>
+  <si>
     <t>A13</t>
   </si>
   <si>
-    <t>NZ</t>
-  </si>
-  <si>
-    <t>avaliador13@teste.com</t>
-  </si>
-  <si>
     <t>Avaliador 14</t>
   </si>
   <si>
+    <t>avaliador14@teste.com</t>
+  </si>
+  <si>
     <t>A14</t>
   </si>
   <si>
-    <t>RG</t>
-  </si>
-  <si>
-    <t>avaliador14@teste.com</t>
-  </si>
-  <si>
     <t>Avaliador 15</t>
   </si>
   <si>
+    <t>avaliador15@teste.com</t>
+  </si>
+  <si>
     <t>A15</t>
   </si>
   <si>
-    <t>SP</t>
-  </si>
-  <si>
-    <t>avaliador15@teste.com</t>
-  </si>
-  <si>
     <t>Avaliador 16</t>
   </si>
   <si>
+    <t>avaliador16@teste.com</t>
+  </si>
+  <si>
     <t>A16</t>
   </si>
   <si>
-    <t>VB</t>
-  </si>
-  <si>
-    <t>avaliador16@teste.com</t>
-  </si>
-  <si>
     <t>Avaliador 17</t>
   </si>
   <si>
+    <t>avaliador17@teste.com</t>
+  </si>
+  <si>
     <t>A17</t>
   </si>
   <si>
-    <t>VG</t>
-  </si>
-  <si>
-    <t>avaliador17@teste.com</t>
-  </si>
-  <si>
     <t>Avaliador 18</t>
   </si>
   <si>
+    <t>avaliador18@teste.com</t>
+  </si>
+  <si>
     <t>A18</t>
   </si>
   <si>
-    <t>VL</t>
-  </si>
-  <si>
-    <t>avaliador18@teste.com</t>
-  </si>
-  <si>
     <t>Avaliador 19</t>
   </si>
   <si>
+    <t>avaliador19@teste.com</t>
+  </si>
+  <si>
     <t>A19</t>
   </si>
   <si>
-    <t>VS</t>
-  </si>
-  <si>
-    <t>avaliador19@teste.com</t>
-  </si>
-  <si>
     <t>Avaliador 20</t>
   </si>
   <si>
+    <t>avaliador20@teste.com</t>
+  </si>
+  <si>
     <t>A20</t>
   </si>
   <si>
-    <t>VK</t>
-  </si>
-  <si>
     <t>Avaliador 21</t>
   </si>
   <si>
+    <t>avaliador21@teste.com</t>
+  </si>
+  <si>
     <t>A21</t>
-  </si>
-  <si>
-    <t>JB</t>
   </si>
   <si>
     <t>CANDIDATOS</t>
@@ -1310,7 +1262,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1367,6 +1319,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
@@ -10204,299 +10159,252 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="10.25"/>
+    <col customWidth="1" min="2" max="2" width="18.5"/>
+    <col customWidth="1" min="3" max="3" width="5.0"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="19" t="s">
         <v>239</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="19" t="s">
         <v>240</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="19" t="s">
         <v>241</v>
       </c>
-      <c r="D1" s="7" t="s">
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="s">
         <v>242</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="s">
+      <c r="B2" s="10" t="s">
         <v>243</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="C2" s="10" t="s">
         <v>244</v>
       </c>
-      <c r="C2" s="7" t="s">
+    </row>
+    <row r="3">
+      <c r="A3" s="10" t="s">
         <v>245</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="B3" s="10" t="s">
         <v>246</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="7" t="s">
+      <c r="C3" s="10" t="s">
         <v>247</v>
       </c>
-      <c r="B3" s="7" t="s">
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="s">
         <v>248</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="B4" s="10" t="s">
         <v>249</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="C4" s="10" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="7" t="s">
+    <row r="5">
+      <c r="A5" s="10" t="s">
         <v>251</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B5" s="10" t="s">
         <v>252</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C5" s="10" t="s">
         <v>253</v>
       </c>
-      <c r="D4" s="7" t="s">
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="s">
         <v>254</v>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="7" t="s">
+      <c r="B6" s="10" t="s">
         <v>255</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="C6" s="10" t="s">
         <v>256</v>
       </c>
-      <c r="C5" s="7" t="s">
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="s">
         <v>257</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="B7" s="10" t="s">
         <v>258</v>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="7" t="s">
+      <c r="C7" s="10" t="s">
         <v>259</v>
       </c>
-      <c r="B6" s="7" t="s">
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="s">
         <v>260</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="B8" s="10" t="s">
         <v>261</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="C8" s="10" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="7" t="s">
+    <row r="9">
+      <c r="A9" s="10" t="s">
         <v>263</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B9" s="10" t="s">
         <v>264</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C9" s="10" t="s">
         <v>265</v>
       </c>
-      <c r="D7" s="7" t="s">
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="s">
         <v>266</v>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="s">
+      <c r="B10" s="10" t="s">
         <v>267</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="C10" s="10" t="s">
         <v>268</v>
       </c>
-      <c r="C8" s="7" t="s">
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="s">
         <v>269</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="B11" s="10" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="s">
+      <c r="C11" s="10" t="s">
         <v>271</v>
       </c>
-      <c r="B9" s="7" t="s">
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="s">
         <v>272</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="B12" s="10" t="s">
         <v>273</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="C12" s="10" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="7" t="s">
+    <row r="13">
+      <c r="A13" s="10" t="s">
         <v>275</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B13" s="10" t="s">
         <v>276</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C13" s="10" t="s">
         <v>277</v>
       </c>
-      <c r="D10" s="7" t="s">
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="s">
         <v>278</v>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="s">
+      <c r="B14" s="10" t="s">
         <v>279</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="C14" s="10" t="s">
         <v>280</v>
       </c>
-      <c r="C11" s="7" t="s">
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="s">
         <v>281</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="B15" s="10" t="s">
         <v>282</v>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="s">
+      <c r="C15" s="10" t="s">
         <v>283</v>
       </c>
-      <c r="B12" s="7" t="s">
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="s">
         <v>284</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="B16" s="10" t="s">
         <v>285</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="C16" s="10" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="7" t="s">
+    <row r="17">
+      <c r="A17" s="10" t="s">
         <v>287</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B17" s="10" t="s">
         <v>288</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C17" s="10" t="s">
         <v>289</v>
       </c>
-      <c r="D13" s="7" t="s">
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="s">
         <v>290</v>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="s">
+      <c r="B18" s="10" t="s">
         <v>291</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="C18" s="10" t="s">
         <v>292</v>
       </c>
-      <c r="C14" s="7" t="s">
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="B19" s="10" t="s">
         <v>294</v>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="s">
+      <c r="C19" s="10" t="s">
         <v>295</v>
       </c>
-      <c r="B15" s="7" t="s">
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="s">
         <v>296</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="B20" s="10" t="s">
         <v>297</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="C20" s="10" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="7" t="s">
+    <row r="21">
+      <c r="A21" s="10" t="s">
         <v>299</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B21" s="10" t="s">
         <v>300</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C21" s="10" t="s">
         <v>301</v>
       </c>
-      <c r="D16" s="7" t="s">
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="s">
         <v>302</v>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="s">
+      <c r="B22" s="10" t="s">
         <v>303</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="C22" s="10" t="s">
         <v>304</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>305</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="7" t="s">
-        <v>307</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>308</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="D18" s="7" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="s">
-        <v>311</v>
-      </c>
-      <c r="B19" s="7" t="s">
-        <v>312</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>313</v>
-      </c>
-      <c r="D19" s="7" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="s">
-        <v>315</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>316</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>317</v>
-      </c>
-      <c r="D20" s="7" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="s">
-        <v>318</v>
-      </c>
-      <c r="B21" s="7" t="s">
-        <v>319</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>320</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>314</v>
       </c>
     </row>
   </sheetData>
@@ -10516,164 +10424,164 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="19" t="s">
-        <v>321</v>
-      </c>
-      <c r="B1" s="20" t="s">
-        <v>322</v>
-      </c>
-      <c r="C1" s="21" t="s">
-        <v>323</v>
-      </c>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
+      <c r="A1" s="20" t="s">
+        <v>305</v>
+      </c>
+      <c r="B1" s="21" t="s">
+        <v>306</v>
+      </c>
+      <c r="C1" s="22" t="s">
+        <v>307</v>
+      </c>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
     </row>
     <row r="2">
       <c r="A2" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="24"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="25"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="25" t="s">
-        <v>308</v>
-      </c>
-      <c r="C3" s="26"/>
+      <c r="B3" s="26" t="s">
+        <v>295</v>
+      </c>
+      <c r="C3" s="27"/>
     </row>
     <row r="4">
       <c r="A4" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="23"/>
-      <c r="C4" s="27"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="28"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="25" t="s">
-        <v>319</v>
-      </c>
-      <c r="C5" s="26"/>
+      <c r="B5" s="26" t="s">
+        <v>304</v>
+      </c>
+      <c r="C5" s="27"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B6" s="23"/>
-      <c r="C6" s="27"/>
+      <c r="B6" s="24"/>
+      <c r="C6" s="28"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B7" s="28"/>
-      <c r="C7" s="26"/>
+      <c r="B7" s="29"/>
+      <c r="C7" s="27"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="29" t="s">
-        <v>284</v>
-      </c>
-      <c r="C8" s="27"/>
+      <c r="B8" s="30" t="s">
+        <v>277</v>
+      </c>
+      <c r="C8" s="28"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="28"/>
-      <c r="C9" s="30" t="s">
-        <v>284</v>
+      <c r="B9" s="29"/>
+      <c r="C9" s="31" t="s">
+        <v>277</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B10" s="29" t="s">
-        <v>308</v>
-      </c>
-      <c r="C10" s="27"/>
+      <c r="B10" s="30" t="s">
+        <v>295</v>
+      </c>
+      <c r="C10" s="28"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B11" s="25" t="s">
-        <v>324</v>
-      </c>
-      <c r="C11" s="30" t="s">
+      <c r="B11" s="26" t="s">
         <v>308</v>
+      </c>
+      <c r="C11" s="31" t="s">
+        <v>295</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B12" s="29" t="s">
-        <v>325</v>
-      </c>
-      <c r="C12" s="31" t="s">
-        <v>264</v>
+      <c r="B12" s="30" t="s">
+        <v>309</v>
+      </c>
+      <c r="C12" s="32" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B13" s="28"/>
-      <c r="C13" s="30" t="s">
-        <v>252</v>
+      <c r="B13" s="29"/>
+      <c r="C13" s="31" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B14" s="23"/>
-      <c r="C14" s="27"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="28"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="B15" s="25" t="s">
-        <v>326</v>
-      </c>
-      <c r="C15" s="30" t="s">
-        <v>327</v>
+      <c r="B15" s="26" t="s">
+        <v>310</v>
+      </c>
+      <c r="C15" s="31" t="s">
+        <v>311</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B16" s="29" t="s">
-        <v>328</v>
-      </c>
-      <c r="C16" s="31" t="s">
-        <v>329</v>
+      <c r="B16" s="30" t="s">
+        <v>312</v>
+      </c>
+      <c r="C16" s="32" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="B17" s="28"/>
-      <c r="C17" s="26"/>
+      <c r="B17" s="29"/>
+      <c r="C17" s="27"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="B18" s="23"/>
-      <c r="C18" s="31" t="s">
+      <c r="B18" s="24"/>
+      <c r="C18" s="32" t="s">
         <v>256</v>
       </c>
     </row>
@@ -10681,93 +10589,93 @@
       <c r="A19" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="B19" s="25" t="s">
-        <v>330</v>
-      </c>
-      <c r="C19" s="26"/>
+      <c r="B19" s="26" t="s">
+        <v>314</v>
+      </c>
+      <c r="C19" s="27"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="B20" s="29" t="s">
-        <v>330</v>
-      </c>
-      <c r="C20" s="31" t="s">
-        <v>248</v>
+      <c r="B20" s="30" t="s">
+        <v>314</v>
+      </c>
+      <c r="C20" s="32" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="B21" s="25" t="s">
-        <v>252</v>
-      </c>
-      <c r="C21" s="26"/>
+      <c r="B21" s="26" t="s">
+        <v>253</v>
+      </c>
+      <c r="C21" s="27"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="B22" s="29" t="s">
-        <v>331</v>
-      </c>
-      <c r="C22" s="27"/>
+      <c r="B22" s="30" t="s">
+        <v>315</v>
+      </c>
+      <c r="C22" s="28"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="B23" s="25" t="s">
-        <v>300</v>
-      </c>
-      <c r="C23" s="30" t="s">
-        <v>304</v>
+      <c r="B23" s="26" t="s">
+        <v>289</v>
+      </c>
+      <c r="C23" s="31" t="s">
+        <v>292</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="B24" s="23"/>
-      <c r="C24" s="27"/>
+      <c r="B24" s="24"/>
+      <c r="C24" s="28"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="B25" s="25" t="s">
-        <v>280</v>
-      </c>
-      <c r="C25" s="30" t="s">
-        <v>304</v>
+      <c r="B25" s="26" t="s">
+        <v>274</v>
+      </c>
+      <c r="C25" s="31" t="s">
+        <v>292</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="B26" s="23"/>
-      <c r="C26" s="31" t="s">
-        <v>264</v>
+      <c r="B26" s="24"/>
+      <c r="C26" s="32" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="B27" s="28"/>
-      <c r="C27" s="26"/>
+      <c r="B27" s="29"/>
+      <c r="C27" s="27"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B28" s="29" t="s">
-        <v>304</v>
-      </c>
-      <c r="C28" s="31" t="s">
+      <c r="B28" s="30" t="s">
+        <v>292</v>
+      </c>
+      <c r="C28" s="32" t="s">
         <v>256</v>
       </c>
     </row>
@@ -10775,75 +10683,75 @@
       <c r="A29" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="B29" s="25" t="s">
-        <v>304</v>
-      </c>
-      <c r="C29" s="30" t="s">
-        <v>280</v>
+      <c r="B29" s="26" t="s">
+        <v>292</v>
+      </c>
+      <c r="C29" s="31" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="B30" s="29" t="s">
-        <v>332</v>
-      </c>
-      <c r="C30" s="27"/>
+      <c r="B30" s="30" t="s">
+        <v>316</v>
+      </c>
+      <c r="C30" s="28"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="B31" s="25" t="s">
-        <v>288</v>
-      </c>
-      <c r="C31" s="30" t="s">
+      <c r="B31" s="26" t="s">
         <v>280</v>
+      </c>
+      <c r="C31" s="31" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="B32" s="23"/>
-      <c r="C32" s="27"/>
+      <c r="B32" s="24"/>
+      <c r="C32" s="28"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="B33" s="28"/>
-      <c r="C33" s="26"/>
+      <c r="B33" s="29"/>
+      <c r="C33" s="27"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="B34" s="29" t="s">
-        <v>304</v>
-      </c>
-      <c r="C34" s="31" t="s">
-        <v>333</v>
+      <c r="B34" s="30" t="s">
+        <v>292</v>
+      </c>
+      <c r="C34" s="32" t="s">
+        <v>317</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="B35" s="25" t="s">
-        <v>264</v>
-      </c>
-      <c r="C35" s="30" t="s">
-        <v>248</v>
+      <c r="B35" s="26" t="s">
+        <v>262</v>
+      </c>
+      <c r="C35" s="31" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="B36" s="23"/>
-      <c r="C36" s="31" t="s">
+      <c r="B36" s="24"/>
+      <c r="C36" s="32" t="s">
         <v>256</v>
       </c>
     </row>
@@ -10851,103 +10759,103 @@
       <c r="A37" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="B37" s="28"/>
-      <c r="C37" s="30" t="s">
-        <v>334</v>
+      <c r="B37" s="29"/>
+      <c r="C37" s="31" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="B38" s="23"/>
-      <c r="C38" s="27"/>
+      <c r="B38" s="24"/>
+      <c r="C38" s="28"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="B39" s="25" t="s">
-        <v>335</v>
-      </c>
-      <c r="C39" s="26"/>
+      <c r="B39" s="26" t="s">
+        <v>319</v>
+      </c>
+      <c r="C39" s="27"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="B40" s="29" t="s">
-        <v>336</v>
-      </c>
-      <c r="C40" s="31" t="s">
-        <v>292</v>
+      <c r="B40" s="30" t="s">
+        <v>320</v>
+      </c>
+      <c r="C40" s="32" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="B41" s="28"/>
-      <c r="C41" s="26"/>
+      <c r="B41" s="29"/>
+      <c r="C41" s="27"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="B42" s="29" t="s">
-        <v>300</v>
-      </c>
-      <c r="C42" s="27"/>
+      <c r="B42" s="30" t="s">
+        <v>289</v>
+      </c>
+      <c r="C42" s="28"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="B43" s="28"/>
-      <c r="C43" s="26"/>
+      <c r="B43" s="29"/>
+      <c r="C43" s="27"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="B44" s="29" t="s">
-        <v>288</v>
-      </c>
-      <c r="C44" s="27"/>
+      <c r="B44" s="30" t="s">
+        <v>280</v>
+      </c>
+      <c r="C44" s="28"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="B45" s="28"/>
-      <c r="C45" s="26"/>
+      <c r="B45" s="29"/>
+      <c r="C45" s="27"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="B46" s="23"/>
-      <c r="C46" s="31" t="s">
-        <v>288</v>
+      <c r="B46" s="24"/>
+      <c r="C46" s="32" t="s">
+        <v>280</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="B47" s="25" t="s">
-        <v>288</v>
-      </c>
-      <c r="C47" s="26"/>
+      <c r="B47" s="26" t="s">
+        <v>280</v>
+      </c>
+      <c r="C47" s="27"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="B48" s="29" t="s">
-        <v>288</v>
-      </c>
-      <c r="C48" s="31" t="s">
+      <c r="B48" s="30" t="s">
+        <v>280</v>
+      </c>
+      <c r="C48" s="32" t="s">
         <v>256</v>
       </c>
     </row>
@@ -10955,466 +10863,466 @@
       <c r="A49" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="B49" s="25" t="s">
-        <v>337</v>
-      </c>
-      <c r="C49" s="26"/>
+      <c r="B49" s="26" t="s">
+        <v>321</v>
+      </c>
+      <c r="C49" s="27"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="B50" s="23"/>
-      <c r="C50" s="27"/>
+      <c r="B50" s="24"/>
+      <c r="C50" s="28"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="B51" s="25" t="s">
-        <v>338</v>
-      </c>
-      <c r="C51" s="30" t="s">
-        <v>304</v>
+      <c r="B51" s="26" t="s">
+        <v>322</v>
+      </c>
+      <c r="C51" s="31" t="s">
+        <v>292</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="B52" s="23"/>
-      <c r="C52" s="31" t="s">
-        <v>339</v>
+      <c r="B52" s="24"/>
+      <c r="C52" s="32" t="s">
+        <v>323</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="B53" s="28"/>
-      <c r="C53" s="26"/>
+      <c r="B53" s="29"/>
+      <c r="C53" s="27"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="B54" s="23"/>
-      <c r="C54" s="27"/>
+      <c r="B54" s="24"/>
+      <c r="C54" s="28"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="B55" s="28"/>
-      <c r="C55" s="30" t="s">
-        <v>288</v>
+      <c r="B55" s="29"/>
+      <c r="C55" s="31" t="s">
+        <v>280</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="B56" s="29" t="s">
+      <c r="B56" s="30" t="s">
         <v>256</v>
       </c>
-      <c r="C56" s="31" t="s">
-        <v>300</v>
+      <c r="C56" s="32" t="s">
+        <v>289</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="B57" s="28"/>
-      <c r="C57" s="26"/>
+      <c r="B57" s="29"/>
+      <c r="C57" s="27"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="s">
         <v>137</v>
       </c>
-      <c r="B58" s="29" t="s">
-        <v>300</v>
-      </c>
-      <c r="C58" s="27"/>
+      <c r="B58" s="30" t="s">
+        <v>289</v>
+      </c>
+      <c r="C58" s="28"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="B59" s="28"/>
-      <c r="C59" s="26"/>
+      <c r="B59" s="29"/>
+      <c r="C59" s="27"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="B60" s="23"/>
-      <c r="C60" s="27"/>
+      <c r="B60" s="24"/>
+      <c r="C60" s="28"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="B61" s="28"/>
-      <c r="C61" s="26"/>
+      <c r="B61" s="29"/>
+      <c r="C61" s="27"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="B62" s="29" t="s">
-        <v>288</v>
-      </c>
-      <c r="C62" s="27"/>
+      <c r="B62" s="30" t="s">
+        <v>280</v>
+      </c>
+      <c r="C62" s="28"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="B63" s="28"/>
-      <c r="C63" s="26"/>
+      <c r="B63" s="29"/>
+      <c r="C63" s="27"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="s">
         <v>149</v>
       </c>
-      <c r="B64" s="23"/>
-      <c r="C64" s="31" t="s">
-        <v>288</v>
+      <c r="B64" s="24"/>
+      <c r="C64" s="32" t="s">
+        <v>280</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="B65" s="28"/>
-      <c r="C65" s="26"/>
+      <c r="B65" s="29"/>
+      <c r="C65" s="27"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="s">
         <v>153</v>
       </c>
-      <c r="B66" s="23"/>
-      <c r="C66" s="31" t="s">
-        <v>288</v>
+      <c r="B66" s="24"/>
+      <c r="C66" s="32" t="s">
+        <v>280</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="B67" s="25" t="s">
-        <v>288</v>
-      </c>
-      <c r="C67" s="30" t="s">
-        <v>240</v>
+      <c r="B67" s="26" t="s">
+        <v>280</v>
+      </c>
+      <c r="C67" s="31" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="7" t="s">
         <v>157</v>
       </c>
-      <c r="B68" s="23"/>
-      <c r="C68" s="27"/>
+      <c r="B68" s="24"/>
+      <c r="C68" s="28"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="B69" s="28"/>
-      <c r="C69" s="26"/>
+      <c r="B69" s="29"/>
+      <c r="C69" s="27"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="B70" s="23"/>
-      <c r="C70" s="27"/>
+      <c r="B70" s="24"/>
+      <c r="C70" s="28"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="B71" s="28"/>
-      <c r="C71" s="26"/>
+      <c r="B71" s="29"/>
+      <c r="C71" s="27"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="B72" s="23"/>
-      <c r="C72" s="27"/>
+      <c r="B72" s="24"/>
+      <c r="C72" s="28"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="B73" s="28"/>
-      <c r="C73" s="26"/>
+      <c r="B73" s="29"/>
+      <c r="C73" s="27"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="B74" s="23"/>
-      <c r="C74" s="27"/>
+      <c r="B74" s="24"/>
+      <c r="C74" s="28"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="B75" s="28"/>
-      <c r="C75" s="26"/>
+      <c r="B75" s="29"/>
+      <c r="C75" s="27"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="B76" s="29" t="s">
+      <c r="B76" s="30" t="s">
+        <v>283</v>
+      </c>
+      <c r="C76" s="32" t="s">
         <v>292</v>
-      </c>
-      <c r="C76" s="31" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="7" t="s">
         <v>175</v>
       </c>
-      <c r="B77" s="28"/>
-      <c r="C77" s="26"/>
+      <c r="B77" s="29"/>
+      <c r="C77" s="27"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="s">
         <v>177</v>
       </c>
-      <c r="B78" s="23"/>
-      <c r="C78" s="27"/>
+      <c r="B78" s="24"/>
+      <c r="C78" s="28"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="s">
         <v>179</v>
       </c>
-      <c r="B79" s="28"/>
-      <c r="C79" s="26"/>
+      <c r="B79" s="29"/>
+      <c r="C79" s="27"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="B80" s="23"/>
-      <c r="C80" s="27"/>
+      <c r="B80" s="24"/>
+      <c r="C80" s="28"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="B81" s="25" t="s">
-        <v>304</v>
-      </c>
-      <c r="C81" s="26"/>
+      <c r="B81" s="26" t="s">
+        <v>292</v>
+      </c>
+      <c r="C81" s="27"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="B82" s="23"/>
-      <c r="C82" s="27"/>
+      <c r="B82" s="24"/>
+      <c r="C82" s="28"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="B83" s="28"/>
-      <c r="C83" s="26"/>
+      <c r="B83" s="29"/>
+      <c r="C83" s="27"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="B84" s="23"/>
-      <c r="C84" s="27"/>
+      <c r="B84" s="24"/>
+      <c r="C84" s="28"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="s">
         <v>191</v>
       </c>
-      <c r="B85" s="28"/>
-      <c r="C85" s="26"/>
+      <c r="B85" s="29"/>
+      <c r="C85" s="27"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="B86" s="23"/>
-      <c r="C86" s="27"/>
+      <c r="B86" s="24"/>
+      <c r="C86" s="28"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="s">
         <v>195</v>
       </c>
-      <c r="B87" s="28"/>
-      <c r="C87" s="30" t="s">
-        <v>304</v>
+      <c r="B87" s="29"/>
+      <c r="C87" s="31" t="s">
+        <v>292</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="B88" s="23"/>
-      <c r="C88" s="27"/>
+      <c r="B88" s="24"/>
+      <c r="C88" s="28"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="B89" s="28"/>
-      <c r="C89" s="26"/>
+      <c r="B89" s="29"/>
+      <c r="C89" s="27"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="B90" s="23"/>
-      <c r="C90" s="27"/>
+      <c r="B90" s="24"/>
+      <c r="C90" s="28"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="s">
         <v>203</v>
       </c>
-      <c r="B91" s="28"/>
-      <c r="C91" s="26"/>
+      <c r="B91" s="29"/>
+      <c r="C91" s="27"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="s">
         <v>205</v>
       </c>
-      <c r="B92" s="23"/>
-      <c r="C92" s="27"/>
+      <c r="B92" s="24"/>
+      <c r="C92" s="28"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="s">
         <v>207</v>
       </c>
-      <c r="B93" s="28"/>
-      <c r="C93" s="26"/>
+      <c r="B93" s="29"/>
+      <c r="C93" s="27"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="s">
         <v>209</v>
       </c>
-      <c r="B94" s="23"/>
-      <c r="C94" s="27"/>
+      <c r="B94" s="24"/>
+      <c r="C94" s="28"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="B95" s="28"/>
-      <c r="C95" s="26"/>
+      <c r="B95" s="29"/>
+      <c r="C95" s="27"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="B96" s="23"/>
-      <c r="C96" s="27"/>
+      <c r="B96" s="24"/>
+      <c r="C96" s="28"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="B97" s="28"/>
-      <c r="C97" s="26"/>
+      <c r="B97" s="29"/>
+      <c r="C97" s="27"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="s">
         <v>217</v>
       </c>
-      <c r="B98" s="29" t="s">
-        <v>339</v>
-      </c>
-      <c r="C98" s="27"/>
+      <c r="B98" s="30" t="s">
+        <v>323</v>
+      </c>
+      <c r="C98" s="28"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="s">
         <v>219</v>
       </c>
-      <c r="B99" s="32" t="s">
-        <v>339</v>
-      </c>
-      <c r="C99" s="28"/>
+      <c r="B99" s="33" t="s">
+        <v>323</v>
+      </c>
+      <c r="C99" s="29"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="B100" s="33"/>
-      <c r="C100" s="23"/>
+      <c r="B100" s="34"/>
+      <c r="C100" s="24"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="s">
         <v>223</v>
       </c>
-      <c r="B101" s="34"/>
-      <c r="C101" s="28"/>
+      <c r="B101" s="35"/>
+      <c r="C101" s="29"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="s">
         <v>225</v>
       </c>
-      <c r="B102" s="33"/>
-      <c r="C102" s="23"/>
+      <c r="B102" s="34"/>
+      <c r="C102" s="24"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="B103" s="34"/>
-      <c r="C103" s="28"/>
+      <c r="B103" s="35"/>
+      <c r="C103" s="29"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="s">
         <v>229</v>
       </c>
-      <c r="B104" s="33"/>
-      <c r="C104" s="23"/>
+      <c r="B104" s="34"/>
+      <c r="C104" s="24"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="B105" s="34"/>
-      <c r="C105" s="28"/>
+      <c r="B105" s="35"/>
+      <c r="C105" s="29"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="s">
         <v>233</v>
       </c>
-      <c r="B106" s="33"/>
-      <c r="C106" s="23"/>
+      <c r="B106" s="34"/>
+      <c r="C106" s="24"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="s">
         <v>235</v>
       </c>
-      <c r="B107" s="32" t="s">
-        <v>300</v>
-      </c>
-      <c r="C107" s="28"/>
+      <c r="B107" s="33" t="s">
+        <v>289</v>
+      </c>
+      <c r="C107" s="29"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="s">
         <v>237</v>
       </c>
-      <c r="B108" s="33"/>
-      <c r="C108" s="23"/>
+      <c r="B108" s="34"/>
+      <c r="C108" s="24"/>
     </row>
     <row r="109">
-      <c r="A109" s="35"/>
-      <c r="B109" s="34"/>
-      <c r="C109" s="28"/>
+      <c r="A109" s="36"/>
+      <c r="B109" s="35"/>
+      <c r="C109" s="29"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>